<commit_message>
M: updated IOR comparision
</commit_message>
<xml_diff>
--- a/results/IOR_MDTest_comparision.xlsx
+++ b/results/IOR_MDTest_comparision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\container-runtime-testing-slurm\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C88A85C-158A-4895-9822-F6482ED58D5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A93E079-3730-48B8-AA74-C3335DFF832D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="12220" xr2:uid="{2FE40472-D93A-4F19-92FD-7FB4454A1223}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="35">
   <si>
     <t>Read Test</t>
   </si>
@@ -126,6 +126,21 @@
   </si>
   <si>
     <t>MD Test (ops/sec)</t>
+  </si>
+  <si>
+    <t>File Read</t>
+  </si>
+  <si>
+    <t>File Removal</t>
+  </si>
+  <si>
+    <t>Tree Creation</t>
+  </si>
+  <si>
+    <t>Tree Removal</t>
+  </si>
+  <si>
+    <t>Mean (ops/sec)</t>
   </si>
 </sst>
 </file>
@@ -161,11 +176,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -500,19 +516,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DC35582-BFC8-4A35-9014-0285CA01C44E}">
-  <dimension ref="A3:S28"/>
+  <dimension ref="A3:Z28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="4" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="10" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.08984375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="11.08984375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="16" max="18" width="11.81640625" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="23" max="26" width="11.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -536,7 +557,7 @@
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -586,7 +607,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -635,8 +656,15 @@
       <c r="S5">
         <v>22.050999999999998</v>
       </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V5" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="W5" s="1"/>
+      <c r="X5" s="1"/>
+      <c r="Y5" s="1"/>
+      <c r="Z5" s="1"/>
+    </row>
+    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -685,8 +713,23 @@
       <c r="S6">
         <v>18.010999999999999</v>
       </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V6" t="s">
+        <v>20</v>
+      </c>
+      <c r="W6" t="s">
+        <v>2</v>
+      </c>
+      <c r="X6" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y6" t="s">
+        <v>3</v>
+      </c>
+      <c r="Z6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -735,8 +778,23 @@
       <c r="S7">
         <v>27.667000000000002</v>
       </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V7" t="s">
+        <v>23</v>
+      </c>
+      <c r="W7">
+        <v>250.827</v>
+      </c>
+      <c r="X7">
+        <v>247.62200000000001</v>
+      </c>
+      <c r="Y7">
+        <v>253.04499999999999</v>
+      </c>
+      <c r="Z7">
+        <v>229.607</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -785,8 +843,23 @@
       <c r="S8">
         <v>20.297999999999998</v>
       </c>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V8" t="s">
+        <v>24</v>
+      </c>
+      <c r="W8" s="2">
+        <v>1321066.362</v>
+      </c>
+      <c r="X8" s="2">
+        <v>1200509.7009999999</v>
+      </c>
+      <c r="Y8" s="2">
+        <v>1181412.622</v>
+      </c>
+      <c r="Z8" s="2">
+        <v>1535211.3859999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -835,8 +908,23 @@
       <c r="S9">
         <v>191079.372</v>
       </c>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V9" t="s">
+        <v>30</v>
+      </c>
+      <c r="W9" s="2">
+        <v>3077.8589999999999</v>
+      </c>
+      <c r="X9" s="2">
+        <v>3133.78</v>
+      </c>
+      <c r="Y9" s="2">
+        <v>3171.1790000000001</v>
+      </c>
+      <c r="Z9" s="2">
+        <v>3092.502</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -885,8 +973,23 @@
       <c r="S10">
         <v>693501.42500000005</v>
       </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V10" t="s">
+        <v>31</v>
+      </c>
+      <c r="W10">
+        <v>234.55</v>
+      </c>
+      <c r="X10">
+        <v>223.19399999999999</v>
+      </c>
+      <c r="Y10">
+        <v>257.34699999999998</v>
+      </c>
+      <c r="Z10">
+        <v>230.18899999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -935,8 +1038,23 @@
       <c r="S11">
         <v>81412.811000000002</v>
       </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V11" t="s">
+        <v>32</v>
+      </c>
+      <c r="W11">
+        <v>12.093</v>
+      </c>
+      <c r="X11">
+        <v>8.2829999999999995</v>
+      </c>
+      <c r="Y11">
+        <v>6.7350000000000003</v>
+      </c>
+      <c r="Z11">
+        <v>11.46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
       <c r="N12" t="s">
         <v>4</v>
       </c>
@@ -955,8 +1073,23 @@
       <c r="S12">
         <v>113182.87300000001</v>
       </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.35">
+      <c r="V12" t="s">
+        <v>33</v>
+      </c>
+      <c r="W12">
+        <v>7.9089999999999998</v>
+      </c>
+      <c r="X12">
+        <v>8.2279999999999998</v>
+      </c>
+      <c r="Y12">
+        <v>9.782</v>
+      </c>
+      <c r="Z12">
+        <v>7.9450000000000003</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
       <c r="N13" t="s">
         <v>2</v>
       </c>
@@ -976,7 +1109,7 @@
         <v>22.48</v>
       </c>
     </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.35">
       <c r="N14" t="s">
         <v>12</v>
       </c>
@@ -996,7 +1129,7 @@
         <v>67.314999999999998</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.35">
       <c r="N15" t="s">
         <v>3</v>
       </c>
@@ -1016,7 +1149,7 @@
         <v>85.679000000000002</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.35">
       <c r="N16" t="s">
         <v>4</v>
       </c>
@@ -1304,10 +1437,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="G3:K3"/>
     <mergeCell ref="N3:S3"/>
+    <mergeCell ref="V5:Z5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>